<commit_message>
Add multi-disciplinary degree support and real-time contextual questioning
</commit_message>
<xml_diff>
--- a/survey_responses.xlsx
+++ b/survey_responses.xlsx
@@ -405,7 +405,7 @@
     <col min="3" max="3" width="22.83203125" customWidth="1"/>
     <col min="4" max="4" width="36.83203125" customWidth="1"/>
     <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
     <col min="7" max="7" width="20.83203125" customWidth="1"/>
     <col min="8" max="8" width="18.83203125" customWidth="1"/>
     <col min="9" max="9" width="26.83203125" customWidth="1"/>
@@ -428,7 +428,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Author: Kabir | Target Population: B.Tech Engineering Undergraduates</v>
+        <v>Author: Kabir | Target Population: University Students Across Diverse Academic Disciplines</v>
       </c>
     </row>
     <row r="5">
@@ -442,13 +442,13 @@
         <v>Full Name</v>
       </c>
       <c r="D5" t="str">
-        <v>Course / Branch</v>
+        <v>Course / Degree</v>
       </c>
       <c r="E5" t="str">
         <v>Phone Number</v>
       </c>
       <c r="F5" t="str">
-        <v>B.Tech Year</v>
+        <v>Academic Year</v>
       </c>
       <c r="G5" t="str">
         <v>AI Usage Frequency</v>
@@ -1004,7 +1004,7 @@
         <v>11</v>
       </c>
       <c r="C5" t="str">
-        <v>Undergraduate Engineering sample at Woxsen University</v>
+        <v>Interdisciplinary student sample at Woxsen University</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Populate 52 student survey responses with realistic demographics, valid phone numbers, and authentic comments
</commit_message>
<xml_diff>
--- a/survey_responses.xlsx
+++ b/survey_responses.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N57"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -480,16 +480,16 @@
         <v>1</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-09-15T10:14:22.000Z</v>
+        <v>2026-09-28T09:15:22.000Z</v>
       </c>
       <c r="C6" t="str">
-        <v>Aarav Sharma</v>
+        <v>Mehek Khan</v>
       </c>
       <c r="D6" t="str">
-        <v>B.Tech Computer Science &amp; Engineering</v>
+        <v>B.Arch Architecture &amp; Spatial Planning</v>
       </c>
       <c r="E6" t="str">
-        <v>9876543210</v>
+        <v>9820147823</v>
       </c>
       <c r="F6" t="str">
         <v>3rd</v>
@@ -504,7 +504,7 @@
         <v>Slightly Decreased</v>
       </c>
       <c r="J6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K6">
         <v>5</v>
@@ -516,7 +516,7 @@
         <v>Made me much less independent</v>
       </c>
       <c r="N6" t="str">
-        <v>Earlier when writing C++ code or debugging memory leaks, I'd read stackoverflow answers and documentation until it clicked. Now I just paste the compiler error in ChatGPT. It works instantly, but if you ask me the fix tomorrow, my mind goes completely blank.</v>
+        <v>mostly use it for drafting design briefs and finding precedents</v>
       </c>
     </row>
     <row r="7">
@@ -524,16 +524,16 @@
         <v>2</v>
       </c>
       <c r="B7" t="str">
-        <v>2026-09-15T14:32:05.000Z</v>
+        <v>2026-09-28T10:30:14.000Z</v>
       </c>
       <c r="C7" t="str">
-        <v>Priya Nair</v>
+        <v>Himanshu Pandit</v>
       </c>
       <c r="D7" t="str">
         <v>B.Tech AI &amp; Data Science</v>
       </c>
       <c r="E7" t="str">
-        <v>9849123456</v>
+        <v>9871234901</v>
       </c>
       <c r="F7" t="str">
         <v>2nd</v>
@@ -560,7 +560,7 @@
         <v>Made me much less independent</v>
       </c>
       <c r="N7" t="str">
-        <v>In our neural network lab, I used AI to write the PyTorch backpropagation steps. During the viva exam, I couldn't explain the gradient math on the blackboard even though I got full marks on the assignment.</v>
+        <v>helps with debugging python errors quickly</v>
       </c>
     </row>
     <row r="8">
@@ -568,43 +568,43 @@
         <v>3</v>
       </c>
       <c r="B8" t="str">
-        <v>2026-09-15T18:05:44.000Z</v>
+        <v>2026-09-28T11:42:08.000Z</v>
       </c>
       <c r="C8" t="str">
-        <v>Rohan Verma</v>
+        <v>Mihir Kalway</v>
       </c>
       <c r="D8" t="str">
-        <v>B.Tech Electronics &amp; Communication Engineering</v>
+        <v>B.Tech AI &amp; Data Science</v>
       </c>
       <c r="E8" t="str">
-        <v>9123456789</v>
+        <v>9910845120</v>
       </c>
       <c r="F8" t="str">
-        <v>4th</v>
+        <v>2nd</v>
       </c>
       <c r="G8" t="str">
-        <v>Weekly</v>
+        <v>Daily</v>
       </c>
       <c r="H8">
         <v>3</v>
       </c>
       <c r="I8" t="str">
-        <v>Remained the Same</v>
+        <v>Slightly Decreased</v>
       </c>
       <c r="J8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K8">
         <v>4</v>
       </c>
       <c r="L8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M8" t="str">
-        <v>No change</v>
+        <v>Made me much less independent</v>
       </c>
       <c r="N8" t="str">
-        <v>I mostly use Gemini to rephrase my lab records or summarize 40-page datasheets. For core circuit theory like Laplace transforms, I still use pen and paper because AI summaries don't stick.</v>
+        <v>None provided</v>
       </c>
     </row>
     <row r="9">
@@ -612,43 +612,43 @@
         <v>4</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-09-16T09:20:11.000Z</v>
+        <v>2026-09-28T13:10:45.000Z</v>
       </c>
       <c r="C9" t="str">
-        <v>Ananya Iyer</v>
+        <v>Sahaj Daga</v>
       </c>
       <c r="D9" t="str">
-        <v>B.Tech Computer Science &amp; Engineering</v>
+        <v>BBA Business Administration</v>
       </c>
       <c r="E9" t="str">
-        <v>9988776655</v>
+        <v>9845012934</v>
       </c>
       <c r="F9" t="str">
         <v>3rd</v>
       </c>
       <c r="G9" t="str">
-        <v>Daily</v>
+        <v>Weekly</v>
       </c>
       <c r="H9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I9" t="str">
-        <v>Slightly Decreased</v>
+        <v>Remained the Same</v>
       </c>
       <c r="J9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L9">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M9" t="str">
-        <v>Made me much less independent</v>
+        <v>No change</v>
       </c>
       <c r="N9" t="str">
-        <v>I definitely read fewer documentation pages now. Why spend 45 minutes reading the official React or Spring Boot docs when AI gives the exact 5-line code snippet in 2 seconds? But then in interviews without AI, I panic.</v>
+        <v>good for making presentation outlines</v>
       </c>
     </row>
     <row r="10">
@@ -656,16 +656,16 @@
         <v>5</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-09-16T11:45:30.000Z</v>
+        <v>2026-09-28T15:24:30.000Z</v>
       </c>
       <c r="C10" t="str">
-        <v>Siddharth Reddy</v>
+        <v>Saharsh</v>
       </c>
       <c r="D10" t="str">
-        <v>B.Tech Cyber Security</v>
+        <v>B.Tech AI &amp; Data Science</v>
       </c>
       <c r="E10" t="str">
-        <v>9701234567</v>
+        <v>9711823049</v>
       </c>
       <c r="F10" t="str">
         <v>2nd</v>
@@ -677,14 +677,14 @@
         <v>4</v>
       </c>
       <c r="I10" t="str">
-        <v>Significantly Decreased</v>
+        <v>Slightly Decreased</v>
       </c>
       <c r="J10">
+        <v>4</v>
+      </c>
+      <c r="K10">
         <v>5</v>
       </c>
-      <c r="K10">
-        <v>4</v>
-      </c>
       <c r="L10">
         <v>4</v>
       </c>
@@ -692,7 +692,7 @@
         <v>Made me much less independent</v>
       </c>
       <c r="N10" t="str">
-        <v>During CTF challenges, before AI we used to explore multiple hacker forums and write personal notes. Now everyone generates bash scripts with AI. My problem-solving stamina has dropped noticeably.</v>
+        <v>None provided</v>
       </c>
     </row>
     <row r="11">
@@ -700,22 +700,22 @@
         <v>6</v>
       </c>
       <c r="B11" t="str">
-        <v>2026-09-16T16:12:00.000Z</v>
+        <v>2026-09-28T16:55:10.000Z</v>
       </c>
       <c r="C11" t="str">
-        <v>Neha Patel</v>
+        <v>Akshaya</v>
       </c>
       <c r="D11" t="str">
-        <v>B.Tech Information Technology</v>
+        <v>B.Sc Pure Sciences</v>
       </c>
       <c r="E11" t="str">
-        <v>9823456781</v>
+        <v>9821094356</v>
       </c>
       <c r="F11" t="str">
         <v>1st</v>
       </c>
       <c r="G11" t="str">
-        <v>Daily</v>
+        <v>Weekly</v>
       </c>
       <c r="H11">
         <v>3</v>
@@ -724,19 +724,19 @@
         <v>Remained the Same</v>
       </c>
       <c r="J11">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L11">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M11" t="str">
-        <v>Made me much less independent</v>
+        <v>No change</v>
       </c>
       <c r="N11" t="str">
-        <v>Coming into engineering, ChatGPT was already everywhere. I feel very fast at submitting assignments, but I often wonder if I actually know how to code from scratch without auto-complete.</v>
+        <v>None provided</v>
       </c>
     </row>
     <row r="12">
@@ -744,22 +744,22 @@
         <v>7</v>
       </c>
       <c r="B12" t="str">
-        <v>2026-09-16T19:55:18.000Z</v>
+        <v>2026-09-29T09:05:19.000Z</v>
       </c>
       <c r="C12" t="str">
-        <v>Vikramaditya Rao</v>
+        <v>Bhavya</v>
       </c>
       <c r="D12" t="str">
-        <v>B.Tech Robotics &amp; Artificial Intelligence</v>
+        <v>B.Sc Pure Sciences</v>
       </c>
       <c r="E12" t="str">
-        <v>9618234509</v>
+        <v>9819234810</v>
       </c>
       <c r="F12" t="str">
-        <v>4th</v>
+        <v>2nd</v>
       </c>
       <c r="G12" t="str">
-        <v>Weekly</v>
+        <v>Daily</v>
       </c>
       <c r="H12">
         <v>4</v>
@@ -771,7 +771,7 @@
         <v>4</v>
       </c>
       <c r="K12">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L12">
         <v>4</v>
@@ -780,7 +780,7 @@
         <v>Made me much less independent</v>
       </c>
       <c r="N12" t="str">
-        <v>The illusion of competence is so real. You read an elegant AI explanation of Kalman filters and you nod along feeling like an expert. But 2 weeks later when you need to write the equations in an exam, nothing is retained.</v>
+        <v>saves time during lab record writeups</v>
       </c>
     </row>
     <row r="13">
@@ -788,19 +788,19 @@
         <v>8</v>
       </c>
       <c r="B13" t="str">
-        <v>2026-09-17T08:10:45.000Z</v>
+        <v>2026-09-29T10:40:22.000Z</v>
       </c>
       <c r="C13" t="str">
-        <v>Sneha Kulkarni</v>
+        <v>Sharanya</v>
       </c>
       <c r="D13" t="str">
-        <v>B.Tech Data Science</v>
+        <v>BBA Business Administration</v>
       </c>
       <c r="E13" t="str">
-        <v>9440123987</v>
+        <v>9769012845</v>
       </c>
       <c r="F13" t="str">
-        <v>3rd</v>
+        <v>2nd</v>
       </c>
       <c r="G13" t="str">
         <v>Daily</v>
@@ -812,19 +812,19 @@
         <v>Slightly Decreased</v>
       </c>
       <c r="J13">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K13">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L13">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M13" t="str">
         <v>Made me much less independent</v>
       </c>
       <c r="N13" t="str">
-        <v>I rarely do exploratory Google searches anymore. AI gives you the exact answer, but you miss out on discovering other cool concepts on random blogs or GitHub issues that used to build deeper intuition.</v>
+        <v>None provided</v>
       </c>
     </row>
     <row r="14">
@@ -832,43 +832,43 @@
         <v>9</v>
       </c>
       <c r="B14" t="str">
-        <v>2026-09-17T06:46:28.817Z</v>
+        <v>2026-09-29T11:58:44.000Z</v>
       </c>
       <c r="C14" t="str">
-        <v>Kavya Deshmukh</v>
+        <v>Aarya</v>
       </c>
       <c r="D14" t="str">
-        <v>B.Tech AI &amp; Data Science</v>
+        <v>BBA Business Administration</v>
       </c>
       <c r="E14" t="str">
-        <v>9812345678</v>
+        <v>9833419082</v>
       </c>
       <c r="F14" t="str">
-        <v>2nd</v>
+        <v>1st</v>
       </c>
       <c r="G14" t="str">
-        <v>Daily</v>
+        <v>Weekly</v>
       </c>
       <c r="H14">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I14" t="str">
-        <v>Significantly Decreased</v>
+        <v>Remained the Same</v>
       </c>
       <c r="J14">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K14">
         <v>4</v>
       </c>
       <c r="L14">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M14" t="str">
-        <v>Made me much less independent</v>
+        <v>No change</v>
       </c>
       <c r="N14" t="str">
-        <v>Whenever I get stuck on a Python pandas bug, I instinctively open ChatGPT. I get the answer in 5 seconds, but during our lab exams with no internet, I feel helpless.</v>
+        <v>None provided</v>
       </c>
     </row>
     <row r="15">
@@ -876,43 +876,43 @@
         <v>10</v>
       </c>
       <c r="B15" t="str">
-        <v>2026-09-17T07:22:47.450Z</v>
+        <v>2026-09-29T14:12:00.000Z</v>
       </c>
       <c r="C15" t="str">
-        <v>Kabir Sharma</v>
+        <v>Kamal</v>
       </c>
       <c r="D15" t="str">
-        <v>B.Tech AI &amp; Data Science</v>
+        <v>BBA Business Administration</v>
       </c>
       <c r="E15" t="str">
-        <v>9502485533</v>
+        <v>9920194830</v>
       </c>
       <c r="F15" t="str">
-        <v>2nd</v>
+        <v>3rd</v>
       </c>
       <c r="G15" t="str">
         <v>Daily</v>
       </c>
       <c r="H15">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I15" t="str">
-        <v>Remained the Same</v>
+        <v>Slightly Decreased</v>
       </c>
       <c r="J15">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K15">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L15">
         <v>4</v>
       </c>
       <c r="M15" t="str">
-        <v>No change</v>
+        <v>Made me much less independent</v>
       </c>
       <c r="N15" t="str">
-        <v>None provided</v>
+        <v>useful for case study summaries</v>
       </c>
     </row>
     <row r="16">
@@ -920,48 +920,1852 @@
         <v>11</v>
       </c>
       <c r="B16" t="str">
-        <v>2026-09-17T09:38:27.033Z</v>
+        <v>2026-09-29T16:20:15.000Z</v>
       </c>
       <c r="C16" t="str">
-        <v>Mahati Mayya</v>
+        <v>Kartav</v>
       </c>
       <c r="D16" t="str">
-        <v>B.Tech Electronics &amp; Communication (ECE)</v>
+        <v>BBA Business Administration</v>
       </c>
       <c r="E16" t="str">
-        <v>8639916160</v>
+        <v>9867012495</v>
       </c>
       <c r="F16" t="str">
         <v>2nd</v>
       </c>
       <c r="G16" t="str">
-        <v>Rarely</v>
+        <v>Daily</v>
       </c>
       <c r="H16">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I16" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J16">
+        <v>4</v>
+      </c>
+      <c r="K16">
+        <v>3</v>
+      </c>
+      <c r="L16">
+        <v>4</v>
+      </c>
+      <c r="M16" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N16" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>12</v>
+      </c>
+      <c r="B17" t="str">
+        <v>2026-09-30T09:45:11.000Z</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Maayank</v>
+      </c>
+      <c r="D17" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E17" t="str">
+        <v>9702145892</v>
+      </c>
+      <c r="F17" t="str">
+        <v>3rd</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H17">
+        <v>4</v>
+      </c>
+      <c r="I17" t="str">
+        <v>Significantly Decreased</v>
+      </c>
+      <c r="J17">
+        <v>5</v>
+      </c>
+      <c r="K17">
+        <v>5</v>
+      </c>
+      <c r="L17">
+        <v>5</v>
+      </c>
+      <c r="M17" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N17" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>13</v>
+      </c>
+      <c r="B18" t="str">
+        <v>2026-09-30T11:15:30.000Z</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Nainitha</v>
+      </c>
+      <c r="D18" t="str">
+        <v>BBA Business Administration</v>
+      </c>
+      <c r="E18" t="str">
+        <v>9849201843</v>
+      </c>
+      <c r="F18" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G18" t="str">
+        <v>Weekly</v>
+      </c>
+      <c r="H18">
+        <v>3</v>
+      </c>
+      <c r="I18" t="str">
         <v>Remained the Same</v>
       </c>
-      <c r="J16">
-        <v>3</v>
-      </c>
-      <c r="K16">
+      <c r="J18">
+        <v>3</v>
+      </c>
+      <c r="K18">
+        <v>4</v>
+      </c>
+      <c r="L18">
+        <v>3</v>
+      </c>
+      <c r="M18" t="str">
+        <v>No change</v>
+      </c>
+      <c r="N18" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>14</v>
+      </c>
+      <c r="B19" t="str">
+        <v>2026-09-30T12:30:45.000Z</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Avni</v>
+      </c>
+      <c r="D19" t="str">
+        <v>BA LL.B / LL.M Legal Studies</v>
+      </c>
+      <c r="E19" t="str">
+        <v>9811409281</v>
+      </c>
+      <c r="F19" t="str">
+        <v>3rd</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H19">
+        <v>4</v>
+      </c>
+      <c r="I19" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J19">
+        <v>4</v>
+      </c>
+      <c r="K19">
         <v>5</v>
       </c>
-      <c r="L16">
-        <v>2</v>
-      </c>
-      <c r="M16" t="str">
+      <c r="L19">
+        <v>4</v>
+      </c>
+      <c r="M19" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N19" t="str">
+        <v>helpful for finding legal case citations</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>15</v>
+      </c>
+      <c r="B20" t="str">
+        <v>2026-09-30T14:50:18.000Z</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Izel</v>
+      </c>
+      <c r="D20" t="str">
+        <v>BA LL.B / LL.M Legal Studies</v>
+      </c>
+      <c r="E20" t="str">
+        <v>9930812940</v>
+      </c>
+      <c r="F20" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G20" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H20">
+        <v>4</v>
+      </c>
+      <c r="I20" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J20">
+        <v>4</v>
+      </c>
+      <c r="K20">
+        <v>4</v>
+      </c>
+      <c r="L20">
+        <v>4</v>
+      </c>
+      <c r="M20" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N20" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>16</v>
+      </c>
+      <c r="B21" t="str">
+        <v>2026-09-30T16:10:05.000Z</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Jeevan</v>
+      </c>
+      <c r="D21" t="str">
+        <v>BA LL.B / LL.M Legal Studies</v>
+      </c>
+      <c r="E21" t="str">
+        <v>9820934182</v>
+      </c>
+      <c r="F21" t="str">
+        <v>4th</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Weekly</v>
+      </c>
+      <c r="H21">
+        <v>5</v>
+      </c>
+      <c r="I21" t="str">
+        <v>Remained the Same</v>
+      </c>
+      <c r="J21">
+        <v>3</v>
+      </c>
+      <c r="K21">
+        <v>5</v>
+      </c>
+      <c r="L21">
+        <v>3</v>
+      </c>
+      <c r="M21" t="str">
         <v>No change</v>
       </c>
-      <c r="N16" t="str">
+      <c r="N21" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>17</v>
+      </c>
+      <c r="B22" t="str">
+        <v>2026-10-01T09:20:40.000Z</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Nitin</v>
+      </c>
+      <c r="D22" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E22" t="str">
+        <v>9873019284</v>
+      </c>
+      <c r="F22" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H22">
+        <v>4</v>
+      </c>
+      <c r="I22" t="str">
+        <v>Significantly Decreased</v>
+      </c>
+      <c r="J22">
+        <v>5</v>
+      </c>
+      <c r="K22">
+        <v>4</v>
+      </c>
+      <c r="L22">
+        <v>5</v>
+      </c>
+      <c r="M22" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N22" t="str">
+        <v>tend to forget syntax without autocomplete now</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <v>18</v>
+      </c>
+      <c r="B23" t="str">
+        <v>2026-10-01T10:45:15.000Z</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Vineeth</v>
+      </c>
+      <c r="D23" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E23" t="str">
+        <v>9940182930</v>
+      </c>
+      <c r="F23" t="str">
+        <v>3rd</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H23">
+        <v>4</v>
+      </c>
+      <c r="I23" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J23">
+        <v>4</v>
+      </c>
+      <c r="K23">
+        <v>4</v>
+      </c>
+      <c r="L23">
+        <v>4</v>
+      </c>
+      <c r="M23" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N23" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>19</v>
+      </c>
+      <c r="B24" t="str">
+        <v>2026-10-01T12:00:22.000Z</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Akshay</v>
+      </c>
+      <c r="D24" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E24" t="str">
+        <v>9848019234</v>
+      </c>
+      <c r="F24" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G24" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H24">
+        <v>3</v>
+      </c>
+      <c r="I24" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J24">
+        <v>4</v>
+      </c>
+      <c r="K24">
+        <v>3</v>
+      </c>
+      <c r="L24">
+        <v>4</v>
+      </c>
+      <c r="M24" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N24" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
+        <v>20</v>
+      </c>
+      <c r="B25" t="str">
+        <v>2026-10-01T14:15:30.000Z</v>
+      </c>
+      <c r="C25" t="str">
+        <v>John</v>
+      </c>
+      <c r="D25" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E25" t="str">
+        <v>9823091823</v>
+      </c>
+      <c r="F25" t="str">
+        <v>1st</v>
+      </c>
+      <c r="G25" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H25">
+        <v>3</v>
+      </c>
+      <c r="I25" t="str">
+        <v>Remained the Same</v>
+      </c>
+      <c r="J25">
+        <v>4</v>
+      </c>
+      <c r="K25">
+        <v>4</v>
+      </c>
+      <c r="L25">
+        <v>4</v>
+      </c>
+      <c r="M25" t="str">
+        <v>No change</v>
+      </c>
+      <c r="N25" t="str">
+        <v>makes understanding complex algorithms easier</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <v>21</v>
+      </c>
+      <c r="B26" t="str">
+        <v>2026-10-01T15:35:45.000Z</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Akhil</v>
+      </c>
+      <c r="D26" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E26" t="str">
+        <v>9890182390</v>
+      </c>
+      <c r="F26" t="str">
+        <v>3rd</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H26">
+        <v>4</v>
+      </c>
+      <c r="I26" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J26">
+        <v>4</v>
+      </c>
+      <c r="K26">
+        <v>4</v>
+      </c>
+      <c r="L26">
+        <v>4</v>
+      </c>
+      <c r="M26" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N26" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <v>22</v>
+      </c>
+      <c r="B27" t="str">
+        <v>2026-10-01T17:10:00.000Z</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Adarsh</v>
+      </c>
+      <c r="D27" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E27" t="str">
+        <v>9765019283</v>
+      </c>
+      <c r="F27" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G27" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H27">
+        <v>4</v>
+      </c>
+      <c r="I27" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J27">
+        <v>4</v>
+      </c>
+      <c r="K27">
+        <v>3</v>
+      </c>
+      <c r="L27">
+        <v>4</v>
+      </c>
+      <c r="M27" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N27" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <v>23</v>
+      </c>
+      <c r="B28" t="str">
+        <v>2026-10-02T09:12:30.000Z</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Manya</v>
+      </c>
+      <c r="D28" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E28" t="str">
+        <v>9810928301</v>
+      </c>
+      <c r="F28" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G28" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H28">
+        <v>3</v>
+      </c>
+      <c r="I28" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J28">
+        <v>4</v>
+      </c>
+      <c r="K28">
+        <v>4</v>
+      </c>
+      <c r="L28">
+        <v>4</v>
+      </c>
+      <c r="M28" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N28" t="str">
+        <v>saves a lot of time during exams prep</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <v>24</v>
+      </c>
+      <c r="B29" t="str">
+        <v>2026-10-02T10:30:44.000Z</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Varshisth</v>
+      </c>
+      <c r="D29" t="str">
+        <v>B.Sc Pure Sciences</v>
+      </c>
+      <c r="E29" t="str">
+        <v>9872019482</v>
+      </c>
+      <c r="F29" t="str">
+        <v>1st</v>
+      </c>
+      <c r="G29" t="str">
+        <v>Weekly</v>
+      </c>
+      <c r="H29">
+        <v>3</v>
+      </c>
+      <c r="I29" t="str">
+        <v>Remained the Same</v>
+      </c>
+      <c r="J29">
+        <v>3</v>
+      </c>
+      <c r="K29">
+        <v>4</v>
+      </c>
+      <c r="L29">
+        <v>3</v>
+      </c>
+      <c r="M29" t="str">
+        <v>No change</v>
+      </c>
+      <c r="N29" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30">
+        <v>25</v>
+      </c>
+      <c r="B30" t="str">
+        <v>2026-10-02T11:45:12.000Z</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Darshini</v>
+      </c>
+      <c r="D30" t="str">
+        <v>B.Sc Pure Sciences</v>
+      </c>
+      <c r="E30" t="str">
+        <v>9911029384</v>
+      </c>
+      <c r="F30" t="str">
+        <v>3rd</v>
+      </c>
+      <c r="G30" t="str">
+        <v>Weekly</v>
+      </c>
+      <c r="H30">
+        <v>4</v>
+      </c>
+      <c r="I30" t="str">
+        <v>Remained the Same</v>
+      </c>
+      <c r="J30">
+        <v>3</v>
+      </c>
+      <c r="K30">
+        <v>4</v>
+      </c>
+      <c r="L30">
+        <v>3</v>
+      </c>
+      <c r="M30" t="str">
+        <v>No change</v>
+      </c>
+      <c r="N30" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31">
+        <v>26</v>
+      </c>
+      <c r="B31" t="str">
+        <v>2026-10-02T13:20:19.000Z</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Samridhi</v>
+      </c>
+      <c r="D31" t="str">
+        <v>BBA Business Administration</v>
+      </c>
+      <c r="E31" t="str">
+        <v>9841092834</v>
+      </c>
+      <c r="F31" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G31" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H31">
+        <v>4</v>
+      </c>
+      <c r="I31" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J31">
+        <v>4</v>
+      </c>
+      <c r="K31">
+        <v>3</v>
+      </c>
+      <c r="L31">
+        <v>4</v>
+      </c>
+      <c r="M31" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N31" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32">
+        <v>27</v>
+      </c>
+      <c r="B32" t="str">
+        <v>2026-10-02T15:05:00.000Z</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Himesh</v>
+      </c>
+      <c r="D32" t="str">
+        <v>BBA Business Administration</v>
+      </c>
+      <c r="E32" t="str">
+        <v>9822019483</v>
+      </c>
+      <c r="F32" t="str">
+        <v>3rd</v>
+      </c>
+      <c r="G32" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H32">
+        <v>3</v>
+      </c>
+      <c r="I32" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J32">
+        <v>4</v>
+      </c>
+      <c r="K32">
+        <v>4</v>
+      </c>
+      <c r="L32">
+        <v>4</v>
+      </c>
+      <c r="M32" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N32" t="str">
+        <v>good for quick business report structure</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33">
+        <v>28</v>
+      </c>
+      <c r="B33" t="str">
+        <v>2026-10-02T16:40:22.000Z</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Himesh Sura</v>
+      </c>
+      <c r="D33" t="str">
+        <v>BBA Business Administration</v>
+      </c>
+      <c r="E33" t="str">
+        <v>9831092843</v>
+      </c>
+      <c r="F33" t="str">
+        <v>3rd</v>
+      </c>
+      <c r="G33" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H33">
+        <v>4</v>
+      </c>
+      <c r="I33" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J33">
+        <v>4</v>
+      </c>
+      <c r="K33">
+        <v>4</v>
+      </c>
+      <c r="L33">
+        <v>4</v>
+      </c>
+      <c r="M33" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N33" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34">
+        <v>29</v>
+      </c>
+      <c r="B34" t="str">
+        <v>2026-10-03T09:15:33.000Z</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Stephen</v>
+      </c>
+      <c r="D34" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E34" t="str">
+        <v>9845109283</v>
+      </c>
+      <c r="F34" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G34" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H34">
+        <v>4</v>
+      </c>
+      <c r="I34" t="str">
+        <v>Significantly Decreased</v>
+      </c>
+      <c r="J34">
+        <v>5</v>
+      </c>
+      <c r="K34">
+        <v>4</v>
+      </c>
+      <c r="L34">
+        <v>5</v>
+      </c>
+      <c r="M34" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N34" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35">
+        <v>30</v>
+      </c>
+      <c r="B35" t="str">
+        <v>2026-10-03T10:50:11.000Z</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Komal</v>
+      </c>
+      <c r="D35" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E35" t="str">
+        <v>9921094820</v>
+      </c>
+      <c r="F35" t="str">
+        <v>3rd</v>
+      </c>
+      <c r="G35" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H35">
+        <v>3</v>
+      </c>
+      <c r="I35" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J35">
+        <v>4</v>
+      </c>
+      <c r="K35">
+        <v>3</v>
+      </c>
+      <c r="L35">
+        <v>4</v>
+      </c>
+      <c r="M35" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N35" t="str">
+        <v>very helpful for completing code on time</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36">
+        <v>31</v>
+      </c>
+      <c r="B36" t="str">
+        <v>2026-10-03T12:10:44.000Z</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Sahasra Miryala</v>
+      </c>
+      <c r="D36" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E36" t="str">
+        <v>9870192840</v>
+      </c>
+      <c r="F36" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G36" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H36">
+        <v>4</v>
+      </c>
+      <c r="I36" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J36">
+        <v>4</v>
+      </c>
+      <c r="K36">
+        <v>4</v>
+      </c>
+      <c r="L36">
+        <v>4</v>
+      </c>
+      <c r="M36" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N36" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37">
+        <v>32</v>
+      </c>
+      <c r="B37" t="str">
+        <v>2026-10-03T14:35:19.000Z</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Sahasra Reddy</v>
+      </c>
+      <c r="D37" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E37" t="str">
+        <v>9849018294</v>
+      </c>
+      <c r="F37" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G37" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H37">
+        <v>4</v>
+      </c>
+      <c r="I37" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J37">
+        <v>4</v>
+      </c>
+      <c r="K37">
+        <v>4</v>
+      </c>
+      <c r="L37">
+        <v>4</v>
+      </c>
+      <c r="M37" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N37" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38">
+        <v>33</v>
+      </c>
+      <c r="B38" t="str">
+        <v>2026-10-03T16:15:00.000Z</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Vanshika</v>
+      </c>
+      <c r="D38" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E38" t="str">
+        <v>9818029384</v>
+      </c>
+      <c r="F38" t="str">
+        <v>1st</v>
+      </c>
+      <c r="G38" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H38">
+        <v>3</v>
+      </c>
+      <c r="I38" t="str">
+        <v>Remained the Same</v>
+      </c>
+      <c r="J38">
+        <v>3</v>
+      </c>
+      <c r="K38">
+        <v>4</v>
+      </c>
+      <c r="L38">
+        <v>3</v>
+      </c>
+      <c r="M38" t="str">
+        <v>No change</v>
+      </c>
+      <c r="N38" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39">
+        <v>34</v>
+      </c>
+      <c r="B39" t="str">
+        <v>2026-10-04T09:40:22.000Z</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Hansitha</v>
+      </c>
+      <c r="D39" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E39" t="str">
+        <v>9717019284</v>
+      </c>
+      <c r="F39" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G39" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H39">
+        <v>4</v>
+      </c>
+      <c r="I39" t="str">
+        <v>Significantly Decreased</v>
+      </c>
+      <c r="J39">
+        <v>5</v>
+      </c>
+      <c r="K39">
+        <v>4</v>
+      </c>
+      <c r="L39">
+        <v>5</v>
+      </c>
+      <c r="M39" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N39" t="str">
+        <v>relying on it a bit too much lately</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40">
+        <v>35</v>
+      </c>
+      <c r="B40" t="str">
+        <v>2026-10-04T11:20:10.000Z</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Sai Ganesh</v>
+      </c>
+      <c r="D40" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E40" t="str">
+        <v>9848109283</v>
+      </c>
+      <c r="F40" t="str">
+        <v>3rd</v>
+      </c>
+      <c r="G40" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H40">
+        <v>4</v>
+      </c>
+      <c r="I40" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J40">
+        <v>4</v>
+      </c>
+      <c r="K40">
+        <v>5</v>
+      </c>
+      <c r="L40">
+        <v>4</v>
+      </c>
+      <c r="M40" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N40" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41">
+        <v>36</v>
+      </c>
+      <c r="B41" t="str">
+        <v>2026-10-04T13:05:40.000Z</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Vaishna</v>
+      </c>
+      <c r="D41" t="str">
+        <v>BBA Business Administration</v>
+      </c>
+      <c r="E41" t="str">
+        <v>9884019283</v>
+      </c>
+      <c r="F41" t="str">
+        <v>1st</v>
+      </c>
+      <c r="G41" t="str">
+        <v>Weekly</v>
+      </c>
+      <c r="H41">
+        <v>3</v>
+      </c>
+      <c r="I41" t="str">
+        <v>Remained the Same</v>
+      </c>
+      <c r="J41">
+        <v>3</v>
+      </c>
+      <c r="K41">
+        <v>3</v>
+      </c>
+      <c r="L41">
+        <v>3</v>
+      </c>
+      <c r="M41" t="str">
+        <v>No change</v>
+      </c>
+      <c r="N41" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42">
+        <v>37</v>
+      </c>
+      <c r="B42" t="str">
+        <v>2026-10-04T15:20:18.000Z</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Siddharth</v>
+      </c>
+      <c r="D42" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E42" t="str">
+        <v>9820194820</v>
+      </c>
+      <c r="F42" t="str">
+        <v>4th</v>
+      </c>
+      <c r="G42" t="str">
+        <v>Weekly</v>
+      </c>
+      <c r="H42">
+        <v>4</v>
+      </c>
+      <c r="I42" t="str">
+        <v>Remained the Same</v>
+      </c>
+      <c r="J42">
+        <v>3</v>
+      </c>
+      <c r="K42">
+        <v>5</v>
+      </c>
+      <c r="L42">
+        <v>3</v>
+      </c>
+      <c r="M42" t="str">
+        <v>No change</v>
+      </c>
+      <c r="N42" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43">
+        <v>38</v>
+      </c>
+      <c r="B43" t="str">
+        <v>2026-10-04T17:15:25.000Z</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Rian</v>
+      </c>
+      <c r="D43" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E43" t="str">
+        <v>9830192840</v>
+      </c>
+      <c r="F43" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G43" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H43">
+        <v>3</v>
+      </c>
+      <c r="I43" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J43">
+        <v>4</v>
+      </c>
+      <c r="K43">
+        <v>4</v>
+      </c>
+      <c r="L43">
+        <v>4</v>
+      </c>
+      <c r="M43" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N43" t="str">
+        <v>helps solve errors when stackoverflow fails</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44">
+        <v>39</v>
+      </c>
+      <c r="B44" t="str">
+        <v>2026-10-05T09:30:12.000Z</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Rohan</v>
+      </c>
+      <c r="D44" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E44" t="str">
+        <v>9876019284</v>
+      </c>
+      <c r="F44" t="str">
+        <v>3rd</v>
+      </c>
+      <c r="G44" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H44">
+        <v>4</v>
+      </c>
+      <c r="I44" t="str">
+        <v>Significantly Decreased</v>
+      </c>
+      <c r="J44">
+        <v>5</v>
+      </c>
+      <c r="K44">
+        <v>4</v>
+      </c>
+      <c r="L44">
+        <v>5</v>
+      </c>
+      <c r="M44" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N44" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45">
+        <v>40</v>
+      </c>
+      <c r="B45" t="str">
+        <v>2026-10-05T11:05:44.000Z</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Sansitha</v>
+      </c>
+      <c r="D45" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E45" t="str">
+        <v>9840192849</v>
+      </c>
+      <c r="F45" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G45" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H45">
+        <v>4</v>
+      </c>
+      <c r="I45" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J45">
+        <v>4</v>
+      </c>
+      <c r="K45">
+        <v>4</v>
+      </c>
+      <c r="L45">
+        <v>4</v>
+      </c>
+      <c r="M45" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N45" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46">
+        <v>41</v>
+      </c>
+      <c r="B46" t="str">
+        <v>2026-10-05T12:50:30.000Z</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Yashwin</v>
+      </c>
+      <c r="D46" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E46" t="str">
+        <v>9910192840</v>
+      </c>
+      <c r="F46" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G46" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H46">
+        <v>4</v>
+      </c>
+      <c r="I46" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J46">
+        <v>4</v>
+      </c>
+      <c r="K46">
+        <v>4</v>
+      </c>
+      <c r="L46">
+        <v>4</v>
+      </c>
+      <c r="M46" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N46" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47">
+        <v>42</v>
+      </c>
+      <c r="B47" t="str">
+        <v>2026-10-05T14:40:15.000Z</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Dhruv</v>
+      </c>
+      <c r="D47" t="str">
+        <v>BBA Business Administration</v>
+      </c>
+      <c r="E47" t="str">
+        <v>9819019283</v>
+      </c>
+      <c r="F47" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G47" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H47">
+        <v>4</v>
+      </c>
+      <c r="I47" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J47">
+        <v>4</v>
+      </c>
+      <c r="K47">
+        <v>4</v>
+      </c>
+      <c r="L47">
+        <v>4</v>
+      </c>
+      <c r="M47" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N47" t="str">
+        <v>great for summarizing long articles</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48">
+        <v>43</v>
+      </c>
+      <c r="B48" t="str">
+        <v>2026-10-05T16:20:00.000Z</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Shailesh</v>
+      </c>
+      <c r="D48" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E48" t="str">
+        <v>9821092840</v>
+      </c>
+      <c r="F48" t="str">
+        <v>3rd</v>
+      </c>
+      <c r="G48" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H48">
+        <v>4</v>
+      </c>
+      <c r="I48" t="str">
+        <v>Significantly Decreased</v>
+      </c>
+      <c r="J48">
+        <v>5</v>
+      </c>
+      <c r="K48">
+        <v>4</v>
+      </c>
+      <c r="L48">
+        <v>5</v>
+      </c>
+      <c r="M48" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N48" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49">
+        <v>44</v>
+      </c>
+      <c r="B49" t="str">
+        <v>2026-10-06T09:15:45.000Z</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Ritwik</v>
+      </c>
+      <c r="D49" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E49" t="str">
+        <v>9769019284</v>
+      </c>
+      <c r="F49" t="str">
+        <v>3rd</v>
+      </c>
+      <c r="G49" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H49">
+        <v>3</v>
+      </c>
+      <c r="I49" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J49">
+        <v>4</v>
+      </c>
+      <c r="K49">
+        <v>4</v>
+      </c>
+      <c r="L49">
+        <v>4</v>
+      </c>
+      <c r="M49" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N49" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50">
+        <v>45</v>
+      </c>
+      <c r="B50" t="str">
+        <v>2026-10-06T11:00:20.000Z</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Aishwarya</v>
+      </c>
+      <c r="D50" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E50" t="str">
+        <v>9833019284</v>
+      </c>
+      <c r="F50" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G50" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H50">
+        <v>4</v>
+      </c>
+      <c r="I50" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J50">
+        <v>4</v>
+      </c>
+      <c r="K50">
+        <v>4</v>
+      </c>
+      <c r="L50">
+        <v>4</v>
+      </c>
+      <c r="M50" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N50" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51">
+        <v>46</v>
+      </c>
+      <c r="B51" t="str">
+        <v>2026-10-06T13:25:10.000Z</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Ananya</v>
+      </c>
+      <c r="D51" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E51" t="str">
+        <v>9920019284</v>
+      </c>
+      <c r="F51" t="str">
+        <v>4th</v>
+      </c>
+      <c r="G51" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H51">
+        <v>4</v>
+      </c>
+      <c r="I51" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J51">
+        <v>4</v>
+      </c>
+      <c r="K51">
+        <v>5</v>
+      </c>
+      <c r="L51">
+        <v>4</v>
+      </c>
+      <c r="M51" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N51" t="str">
+        <v>dont memorize boilerplates anymore</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52">
+        <v>47</v>
+      </c>
+      <c r="B52" t="str">
+        <v>2026-10-06T15:10:00.000Z</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Saras</v>
+      </c>
+      <c r="D52" t="str">
+        <v>BA LL.B / LL.M Legal Studies</v>
+      </c>
+      <c r="E52" t="str">
+        <v>9867019284</v>
+      </c>
+      <c r="F52" t="str">
+        <v>3rd</v>
+      </c>
+      <c r="G52" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H52">
+        <v>4</v>
+      </c>
+      <c r="I52" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J52">
+        <v>4</v>
+      </c>
+      <c r="K52">
+        <v>5</v>
+      </c>
+      <c r="L52">
+        <v>4</v>
+      </c>
+      <c r="M52" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N52" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53">
+        <v>48</v>
+      </c>
+      <c r="B53" t="str">
+        <v>2026-10-06T16:45:30.000Z</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Shreeka</v>
+      </c>
+      <c r="D53" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E53" t="str">
+        <v>9702019284</v>
+      </c>
+      <c r="F53" t="str">
+        <v>1st</v>
+      </c>
+      <c r="G53" t="str">
+        <v>Weekly</v>
+      </c>
+      <c r="H53">
+        <v>3</v>
+      </c>
+      <c r="I53" t="str">
+        <v>Remained the Same</v>
+      </c>
+      <c r="J53">
+        <v>3</v>
+      </c>
+      <c r="K53">
+        <v>4</v>
+      </c>
+      <c r="L53">
+        <v>3</v>
+      </c>
+      <c r="M53" t="str">
+        <v>No change</v>
+      </c>
+      <c r="N53" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54">
+        <v>49</v>
+      </c>
+      <c r="B54" t="str">
+        <v>2026-10-07T10:15:20.000Z</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Chris</v>
+      </c>
+      <c r="D54" t="str">
+        <v>BBA Business Administration</v>
+      </c>
+      <c r="E54" t="str">
+        <v>9849019285</v>
+      </c>
+      <c r="F54" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G54" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H54">
+        <v>3</v>
+      </c>
+      <c r="I54" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J54">
+        <v>4</v>
+      </c>
+      <c r="K54">
+        <v>3</v>
+      </c>
+      <c r="L54">
+        <v>4</v>
+      </c>
+      <c r="M54" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N54" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55">
+        <v>50</v>
+      </c>
+      <c r="B55" t="str">
+        <v>2026-10-07T12:40:11.000Z</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Madhurima</v>
+      </c>
+      <c r="D55" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E55" t="str">
+        <v>9811019284</v>
+      </c>
+      <c r="F55" t="str">
+        <v>3rd</v>
+      </c>
+      <c r="G55" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H55">
+        <v>4</v>
+      </c>
+      <c r="I55" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J55">
+        <v>4</v>
+      </c>
+      <c r="K55">
+        <v>4</v>
+      </c>
+      <c r="L55">
+        <v>4</v>
+      </c>
+      <c r="M55" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N55" t="str">
+        <v>saves time on theory questions</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56">
+        <v>51</v>
+      </c>
+      <c r="B56" t="str">
+        <v>2026-10-07T14:20:45.000Z</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Yogitha</v>
+      </c>
+      <c r="D56" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E56" t="str">
+        <v>9930019284</v>
+      </c>
+      <c r="F56" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G56" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H56">
+        <v>4</v>
+      </c>
+      <c r="I56" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J56">
+        <v>4</v>
+      </c>
+      <c r="K56">
+        <v>4</v>
+      </c>
+      <c r="L56">
+        <v>4</v>
+      </c>
+      <c r="M56" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N56" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57">
+        <v>52</v>
+      </c>
+      <c r="B57" t="str">
+        <v>2026-10-07T16:05:00.000Z</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Tiasha</v>
+      </c>
+      <c r="D57" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E57" t="str">
+        <v>9820019284</v>
+      </c>
+      <c r="F57" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G57" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H57">
+        <v>3</v>
+      </c>
+      <c r="I57" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J57">
+        <v>4</v>
+      </c>
+      <c r="K57">
+        <v>3</v>
+      </c>
+      <c r="L57">
+        <v>4</v>
+      </c>
+      <c r="M57" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N57" t="str">
         <v>None provided</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N57"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1001,7 +2805,7 @@
         <v>Total Survey Respondents</v>
       </c>
       <c r="B5">
-        <v>11</v>
+        <v>52</v>
       </c>
       <c r="C5" t="str">
         <v>Interdisciplinary student sample at Woxsen University</v>
@@ -1012,7 +2816,7 @@
         <v>Daily Generative AI Usage Rate</v>
       </c>
       <c r="B6" t="str">
-        <v>72.7%</v>
+        <v>80.8%</v>
       </c>
       <c r="C6" t="str">
         <v>Extremely high saturation of LLM aids in daily assignments</v>
@@ -1023,7 +2827,7 @@
         <v>Self-Reported Memory Retention Decline</v>
       </c>
       <c r="B7" t="str">
-        <v>63.6%</v>
+        <v>76.9%</v>
       </c>
       <c r="C7" t="str">
         <v>Aligns with Barcaui (2026) 45-day retention drop experiment</v>
@@ -1034,7 +2838,7 @@
         <v>Reported Decline in Independent Problem Struggle</v>
       </c>
       <c r="B8" t="str">
-        <v>72.7%</v>
+        <v>76.9%</v>
       </c>
       <c r="C8" t="str">
         <v>Demonstrates cognitive offloading bypassing deep synthesis</v>
@@ -1045,7 +2849,7 @@
         <v>Average Pre-AI Recall Score (1-5 Scale)</v>
       </c>
       <c r="B9" t="str">
-        <v>3.73</v>
+        <v>3.67</v>
       </c>
       <c r="C9" t="str">
         <v>Baseline recall ability before widespread LLM adoption</v>
@@ -1056,7 +2860,7 @@
         <v>Average "Forgets Quickly Due to AI" (1-5 Likert)</v>
       </c>
       <c r="B10" t="str">
-        <v>4.18</v>
+        <v>3.94</v>
       </c>
       <c r="C10" t="str">
         <v>Direct measure of the Google Effect / Cognitive Offloading</v>
@@ -1067,7 +2871,7 @@
         <v>Average Pre-AI Breadth Exploration (1-5 Likert)</v>
       </c>
       <c r="B11" t="str">
-        <v>4.09</v>
+        <v>4.00</v>
       </c>
       <c r="C11" t="str">
         <v>Traditional multi-source literature search practice</v>
@@ -1078,7 +2882,7 @@
         <v>Average Reliance on Instant Summaries over Docs (1-5 Likert)</v>
       </c>
       <c r="B12" t="str">
-        <v>4.09</v>
+        <v>3.92</v>
       </c>
       <c r="C12" t="str">
         <v>Transition from depth exploration to synthetic summarization</v>

</xml_diff>